<commit_message>
chore(data): update real_time_sales_with_platform dataset
</commit_message>
<xml_diff>
--- a/data/real_time_sales_with_platform.xlsx
+++ b/data/real_time_sales_with_platform.xlsx
@@ -1,41 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_28AB0574DD864ED432C07777A760BE9BCAFA136B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A525DB4F-8728-4A4D-AA55-E00F8C5BF598}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Real-Time Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Summary Dashboard" sheetId="2" r:id="rId2"/>
+    <sheet r:id="rId1" name="Real-Time Data" sheetId="1"/>
+    <sheet r:id="rId2" name="Summary Dashboard" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Real-Time Data'!$A$1:$F$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Real-Time Data'!$A$1:$F$121</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>platform</t>
   </si>
@@ -172,27 +176,31 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="171" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="11"/>
+      <color auto="1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -206,25 +214,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2A363B"/>
-        <bgColor rgb="FF2A363B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7F9F9"/>
-        <bgColor rgb="FFF7F9F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E434C"/>
-        <bgColor rgb="FF1E434C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAECEE"/>
-        <bgColor rgb="FFEAECEE"/>
       </patternFill>
     </fill>
   </fills>
@@ -257,54 +261,68 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="3" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="2" fillId="5" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -591,19 +609,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{65F0804B-A243-48E4-A37E-44095C0224D3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:F121"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="1" max="1" width="15.00390625" customWidth="1"/>
+    <col min="2" max="2" width="20.00390625" customWidth="1"/>
+    <col min="3" max="3" width="18.00390625" customWidth="1"/>
+    <col min="4" max="4" width="12.00390625" customWidth="1"/>
+    <col min="5" max="5" width="18.00390625" customWidth="1"/>
+    <col min="6" max="6" width="15.00390625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -623,7 +641,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -643,7 +661,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
@@ -663,7 +681,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -677,13 +695,13 @@
         <v>9</v>
       </c>
       <c r="E4" s="3">
-        <v>20162.740000000002</v>
+        <v>20162.74</v>
       </c>
       <c r="F4" s="4">
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
@@ -703,7 +721,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
@@ -723,7 +741,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -743,7 +761,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -757,13 +775,13 @@
         <v>16</v>
       </c>
       <c r="E8" s="3">
-        <v>34120.160000000003</v>
+        <v>34120.16</v>
       </c>
       <c r="F8" s="4">
         <v>461</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="5" t="s">
         <v>6</v>
       </c>
@@ -783,7 +801,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -803,7 +821,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -823,7 +841,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
@@ -843,7 +861,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="5" t="s">
         <v>6</v>
       </c>
@@ -863,7 +881,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -883,7 +901,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
@@ -903,7 +921,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -923,7 +941,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="5" t="s">
         <v>6</v>
       </c>
@@ -943,7 +961,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>6</v>
       </c>
@@ -963,7 +981,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="5" t="s">
         <v>6</v>
       </c>
@@ -983,7 +1001,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
@@ -1003,7 +1021,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="5" t="s">
         <v>14</v>
       </c>
@@ -1023,7 +1041,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>6</v>
       </c>
@@ -1037,13 +1055,13 @@
         <v>19</v>
       </c>
       <c r="E22" s="3">
-        <v>37673.879999999997</v>
+        <v>37673.88</v>
       </c>
       <c r="F22" s="4">
         <v>704</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" ht="15" customHeight="1">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
@@ -1063,7 +1081,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>6</v>
       </c>
@@ -1077,13 +1095,13 @@
         <v>19</v>
       </c>
       <c r="E24" s="3">
-        <v>16393.580000000002</v>
+        <v>16393.58</v>
       </c>
       <c r="F24" s="4">
         <v>260</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" ht="15" customHeight="1">
       <c r="A25" s="5" t="s">
         <v>10</v>
       </c>
@@ -1103,7 +1121,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>14</v>
       </c>
@@ -1123,7 +1141,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" ht="15" customHeight="1">
       <c r="A27" s="5" t="s">
         <v>6</v>
       </c>
@@ -1143,7 +1161,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" ht="15" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>10</v>
       </c>
@@ -1157,13 +1175,13 @@
         <v>20</v>
       </c>
       <c r="E28" s="3">
-        <v>17469.810000000001</v>
+        <v>17469.81</v>
       </c>
       <c r="F28" s="4">
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" ht="15" customHeight="1">
       <c r="A29" s="5" t="s">
         <v>14</v>
       </c>
@@ -1183,7 +1201,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" ht="15" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>14</v>
       </c>
@@ -1203,7 +1221,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" ht="15" customHeight="1">
       <c r="A31" s="5" t="s">
         <v>14</v>
       </c>
@@ -1223,7 +1241,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>6</v>
       </c>
@@ -1243,7 +1261,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" ht="15" customHeight="1">
       <c r="A33" s="5" t="s">
         <v>6</v>
       </c>
@@ -1263,7 +1281,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" ht="15" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>6</v>
       </c>
@@ -1283,7 +1301,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" ht="15" customHeight="1">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -1303,7 +1321,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" ht="15" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>14</v>
       </c>
@@ -1323,7 +1341,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" ht="15" customHeight="1">
       <c r="A37" s="5" t="s">
         <v>6</v>
       </c>
@@ -1343,7 +1361,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" ht="15" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>6</v>
       </c>
@@ -1363,7 +1381,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" ht="15" customHeight="1">
       <c r="A39" s="5" t="s">
         <v>10</v>
       </c>
@@ -1383,7 +1401,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" ht="15" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>10</v>
       </c>
@@ -1403,7 +1421,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" ht="15" customHeight="1">
       <c r="A41" s="5" t="s">
         <v>14</v>
       </c>
@@ -1423,7 +1441,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" ht="15" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1443,7 +1461,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" ht="15" customHeight="1">
       <c r="A43" s="5" t="s">
         <v>10</v>
       </c>
@@ -1463,7 +1481,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" ht="15" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>10</v>
       </c>
@@ -1483,7 +1501,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" ht="15" customHeight="1">
       <c r="A45" s="5" t="s">
         <v>14</v>
       </c>
@@ -1503,7 +1521,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" ht="15" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>14</v>
       </c>
@@ -1523,7 +1541,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" ht="15" customHeight="1">
       <c r="A47" s="5" t="s">
         <v>6</v>
       </c>
@@ -1543,7 +1561,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" ht="15" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>6</v>
       </c>
@@ -1563,7 +1581,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" ht="15" customHeight="1">
       <c r="A49" s="5" t="s">
         <v>6</v>
       </c>
@@ -1583,7 +1601,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" ht="15" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>10</v>
       </c>
@@ -1603,7 +1621,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" ht="15" customHeight="1">
       <c r="A51" s="5" t="s">
         <v>14</v>
       </c>
@@ -1623,7 +1641,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" ht="15" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>6</v>
       </c>
@@ -1643,7 +1661,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" ht="15" customHeight="1">
       <c r="A53" s="5" t="s">
         <v>10</v>
       </c>
@@ -1663,7 +1681,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" ht="15" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>10</v>
       </c>
@@ -1683,7 +1701,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" ht="15" customHeight="1">
       <c r="A55" s="5" t="s">
         <v>10</v>
       </c>
@@ -1703,7 +1721,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" ht="15" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>10</v>
       </c>
@@ -1723,7 +1741,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" ht="15" customHeight="1">
       <c r="A57" s="5" t="s">
         <v>10</v>
       </c>
@@ -1743,7 +1761,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" ht="15" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>10</v>
       </c>
@@ -1763,7 +1781,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" ht="15" customHeight="1">
       <c r="A59" s="5" t="s">
         <v>14</v>
       </c>
@@ -1783,7 +1801,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" ht="15" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>14</v>
       </c>
@@ -1803,7 +1821,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" ht="15" customHeight="1">
       <c r="A61" s="5" t="s">
         <v>14</v>
       </c>
@@ -1817,13 +1835,13 @@
         <v>26</v>
       </c>
       <c r="E61" s="6">
-        <v>72032.009999999995</v>
+        <v>72032.01</v>
       </c>
       <c r="F61" s="7">
         <v>437</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" ht="15" customHeight="1">
       <c r="A62" s="2" t="s">
         <v>6</v>
       </c>
@@ -1837,13 +1855,13 @@
         <v>27</v>
       </c>
       <c r="E62" s="3">
-        <v>52831.839999999997</v>
+        <v>52831.84</v>
       </c>
       <c r="F62" s="4">
         <v>298</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" ht="15" customHeight="1">
       <c r="A63" s="5" t="s">
         <v>6</v>
       </c>
@@ -1857,13 +1875,13 @@
         <v>27</v>
       </c>
       <c r="E63" s="6">
-        <v>38514.620000000003</v>
+        <v>38514.62</v>
       </c>
       <c r="F63" s="7">
         <v>613</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" ht="15" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>10</v>
       </c>
@@ -1883,7 +1901,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" ht="15" customHeight="1">
       <c r="A65" s="5" t="s">
         <v>10</v>
       </c>
@@ -1903,7 +1921,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" ht="15" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>10</v>
       </c>
@@ -1923,7 +1941,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" ht="15" customHeight="1">
       <c r="A67" s="5" t="s">
         <v>6</v>
       </c>
@@ -1937,13 +1955,13 @@
         <v>28</v>
       </c>
       <c r="E67" s="6">
-        <v>57045.120000000003</v>
+        <v>57045.12</v>
       </c>
       <c r="F67" s="7">
         <v>511</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" ht="15" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>10</v>
       </c>
@@ -1963,7 +1981,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" ht="15" customHeight="1">
       <c r="A69" s="5" t="s">
         <v>14</v>
       </c>
@@ -1983,7 +2001,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" ht="15" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>14</v>
       </c>
@@ -2003,7 +2021,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" ht="15" customHeight="1">
       <c r="A71" s="5" t="s">
         <v>14</v>
       </c>
@@ -2023,7 +2041,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" ht="15" customHeight="1">
       <c r="A72" s="2" t="s">
         <v>6</v>
       </c>
@@ -2037,13 +2055,13 @@
         <v>29</v>
       </c>
       <c r="E72" s="3">
-        <v>27477.759999999998</v>
+        <v>27477.76</v>
       </c>
       <c r="F72" s="4">
         <v>358</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" ht="15" customHeight="1">
       <c r="A73" s="5" t="s">
         <v>14</v>
       </c>
@@ -2063,7 +2081,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" ht="15" customHeight="1">
       <c r="A74" s="2" t="s">
         <v>14</v>
       </c>
@@ -2083,7 +2101,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" ht="15" customHeight="1">
       <c r="A75" s="5" t="s">
         <v>14</v>
       </c>
@@ -2103,7 +2121,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" ht="15" customHeight="1">
       <c r="A76" s="2" t="s">
         <v>14</v>
       </c>
@@ -2123,7 +2141,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" ht="15" customHeight="1">
       <c r="A77" s="5" t="s">
         <v>6</v>
       </c>
@@ -2143,7 +2161,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" ht="15" customHeight="1">
       <c r="A78" s="2" t="s">
         <v>6</v>
       </c>
@@ -2163,7 +2181,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" ht="15" customHeight="1">
       <c r="A79" s="5" t="s">
         <v>6</v>
       </c>
@@ -2183,7 +2201,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" ht="15" customHeight="1">
       <c r="A80" s="2" t="s">
         <v>10</v>
       </c>
@@ -2203,7 +2221,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" ht="15" customHeight="1">
       <c r="A81" s="5" t="s">
         <v>14</v>
       </c>
@@ -2223,7 +2241,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" ht="15" customHeight="1">
       <c r="A82" s="2" t="s">
         <v>6</v>
       </c>
@@ -2243,7 +2261,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" ht="15" customHeight="1">
       <c r="A83" s="5" t="s">
         <v>10</v>
       </c>
@@ -2263,7 +2281,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" ht="15" customHeight="1">
       <c r="A84" s="2" t="s">
         <v>10</v>
       </c>
@@ -2283,7 +2301,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" ht="15" customHeight="1">
       <c r="A85" s="5" t="s">
         <v>10</v>
       </c>
@@ -2303,7 +2321,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" ht="15" customHeight="1">
       <c r="A86" s="2" t="s">
         <v>14</v>
       </c>
@@ -2323,7 +2341,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" ht="15" customHeight="1">
       <c r="A87" s="5" t="s">
         <v>6</v>
       </c>
@@ -2343,7 +2361,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" ht="15" customHeight="1">
       <c r="A88" s="2" t="s">
         <v>6</v>
       </c>
@@ -2363,7 +2381,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" ht="15" customHeight="1">
       <c r="A89" s="5" t="s">
         <v>14</v>
       </c>
@@ -2383,7 +2401,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" ht="15" customHeight="1">
       <c r="A90" s="2" t="s">
         <v>14</v>
       </c>
@@ -2403,7 +2421,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" ht="15" customHeight="1">
       <c r="A91" s="5" t="s">
         <v>14</v>
       </c>
@@ -2423,7 +2441,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" ht="15" customHeight="1">
       <c r="A92" s="2" t="s">
         <v>6</v>
       </c>
@@ -2443,7 +2461,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" ht="15" customHeight="1">
       <c r="A93" s="5" t="s">
         <v>6</v>
       </c>
@@ -2463,7 +2481,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" ht="15" customHeight="1">
       <c r="A94" s="2" t="s">
         <v>10</v>
       </c>
@@ -2483,7 +2501,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" ht="15" customHeight="1">
       <c r="A95" s="5" t="s">
         <v>10</v>
       </c>
@@ -2503,7 +2521,7 @@
         <v>1120</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" ht="15" customHeight="1">
       <c r="A96" s="2" t="s">
         <v>14</v>
       </c>
@@ -2517,13 +2535,13 @@
         <v>33</v>
       </c>
       <c r="E96" s="3">
-        <v>37575.839999999997</v>
+        <v>37575.84</v>
       </c>
       <c r="F96" s="4">
         <v>337</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" ht="15" customHeight="1">
       <c r="A97" s="5" t="s">
         <v>6</v>
       </c>
@@ -2543,7 +2561,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" ht="15" customHeight="1">
       <c r="A98" s="2" t="s">
         <v>10</v>
       </c>
@@ -2563,7 +2581,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" ht="15" customHeight="1">
       <c r="A99" s="5" t="s">
         <v>10</v>
       </c>
@@ -2583,7 +2601,7 @@
         <v>1227</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" ht="15" customHeight="1">
       <c r="A100" s="2" t="s">
         <v>14</v>
       </c>
@@ -2603,7 +2621,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" ht="15" customHeight="1">
       <c r="A101" s="5" t="s">
         <v>14</v>
       </c>
@@ -2623,7 +2641,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" ht="15" customHeight="1">
       <c r="A102" s="2" t="s">
         <v>10</v>
       </c>
@@ -2643,7 +2661,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" ht="15" customHeight="1">
       <c r="A103" s="5" t="s">
         <v>10</v>
       </c>
@@ -2663,7 +2681,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" ht="15" customHeight="1">
       <c r="A104" s="2" t="s">
         <v>10</v>
       </c>
@@ -2683,7 +2701,7 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" ht="15" customHeight="1">
       <c r="A105" s="5" t="s">
         <v>10</v>
       </c>
@@ -2703,7 +2721,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" ht="15" customHeight="1">
       <c r="A106" s="2" t="s">
         <v>14</v>
       </c>
@@ -2723,7 +2741,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" ht="15" customHeight="1">
       <c r="A107" s="5" t="s">
         <v>6</v>
       </c>
@@ -2743,7 +2761,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" ht="15" customHeight="1">
       <c r="A108" s="2" t="s">
         <v>10</v>
       </c>
@@ -2763,7 +2781,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" ht="15" customHeight="1">
       <c r="A109" s="5" t="s">
         <v>10</v>
       </c>
@@ -2783,7 +2801,7 @@
         <v>1120</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" ht="15" customHeight="1">
       <c r="A110" s="2" t="s">
         <v>10</v>
       </c>
@@ -2803,7 +2821,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" ht="15" customHeight="1">
       <c r="A111" s="5" t="s">
         <v>10</v>
       </c>
@@ -2823,7 +2841,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" ht="15" customHeight="1">
       <c r="A112" s="2" t="s">
         <v>6</v>
       </c>
@@ -2837,13 +2855,13 @@
         <v>37</v>
       </c>
       <c r="E112" s="3">
-        <v>49784.480000000003</v>
+        <v>49784.48</v>
       </c>
       <c r="F112" s="4">
         <v>252</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" ht="15" customHeight="1">
       <c r="A113" s="5" t="s">
         <v>10</v>
       </c>
@@ -2863,7 +2881,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" ht="15" customHeight="1">
       <c r="A114" s="2" t="s">
         <v>14</v>
       </c>
@@ -2883,7 +2901,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" ht="15" customHeight="1">
       <c r="A115" s="5" t="s">
         <v>14</v>
       </c>
@@ -2903,7 +2921,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" ht="15" customHeight="1">
       <c r="A116" s="2" t="s">
         <v>14</v>
       </c>
@@ -2923,7 +2941,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" ht="15" customHeight="1">
       <c r="A117" s="5" t="s">
         <v>10</v>
       </c>
@@ -2943,7 +2961,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" ht="15" customHeight="1">
       <c r="A118" s="2" t="s">
         <v>10</v>
       </c>
@@ -2957,13 +2975,13 @@
         <v>38</v>
       </c>
       <c r="E118" s="3">
-        <v>67570.080000000002</v>
+        <v>67570.08</v>
       </c>
       <c r="F118" s="4">
         <v>434</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" ht="15" customHeight="1">
       <c r="A119" s="5" t="s">
         <v>10</v>
       </c>
@@ -2983,7 +3001,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" ht="15" customHeight="1">
       <c r="A120" s="2" t="s">
         <v>14</v>
       </c>
@@ -3003,7 +3021,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" ht="15" customHeight="1">
       <c r="A121" s="5" t="s">
         <v>14</v>
       </c>
@@ -3017,30 +3035,37 @@
         <v>38</v>
       </c>
       <c r="E121" s="6">
-        <v>95039.679999999993</v>
+        <v>95039.68</v>
       </c>
       <c r="F121" s="7">
         <v>517</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F121" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F121"/>
+  <printOptions/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{20FCB4B3-E149-411C-9D7D-317754F71609}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="1" max="1" width="15.00390625" customWidth="1"/>
+    <col min="2" max="2" width="25.00390625" customWidth="1"/>
+    <col min="3" max="3" width="20.00390625" customWidth="1"/>
+    <col min="4" max="4" width="18.00390625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>39</v>
       </c>
@@ -3054,7 +3079,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -3068,7 +3093,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
@@ -3076,13 +3101,13 @@
         <v>12</v>
       </c>
       <c r="C3" s="6">
-        <v>663528.80000000005</v>
+        <v>663528.8</v>
       </c>
       <c r="D3" s="7">
         <v>6202</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -3096,7 +3121,7 @@
         <v>4160</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -3110,7 +3135,7 @@
         <v>2489</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
@@ -3118,13 +3143,13 @@
         <v>7</v>
       </c>
       <c r="C6" s="6">
-        <v>629072.06999999995</v>
+        <v>629072.07</v>
       </c>
       <c r="D6" s="7">
         <v>4364</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -3138,7 +3163,7 @@
         <v>3655</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
@@ -3146,13 +3171,13 @@
         <v>12</v>
       </c>
       <c r="C8" s="6">
-        <v>687092.57000000007</v>
+        <v>687092.5700000001</v>
       </c>
       <c r="D8" s="7">
         <v>4117</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -3166,7 +3191,7 @@
         <v>4077</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -3180,7 +3205,7 @@
         <v>4855</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
@@ -3188,13 +3213,13 @@
         <v>7</v>
       </c>
       <c r="C11" s="6">
-        <v>548535.31000000006</v>
+        <v>548535.31</v>
       </c>
       <c r="D11" s="7">
         <v>4102</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
@@ -3208,7 +3233,7 @@
         <v>3961</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
@@ -3222,7 +3247,7 @@
         <v>2685</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
@@ -3236,7 +3261,7 @@
         <v>2642</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
@@ -3250,7 +3275,7 @@
         <v>5713</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="5" t="s">
         <v>14</v>
       </c>
@@ -3264,21 +3289,28 @@
         <v>4378</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="9" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="10">
-        <f>SUM(C2:C16)</f>
+        <f t="shared" si="0" ref="C17:D17">SUM(C2:C16)</f>
         <v>7244101.25</v>
       </c>
       <c r="D17" s="11">
-        <f>SUM(D2:D16)</f>
+        <f t="shared" si="0"/>
         <v>58967</v>
       </c>
     </row>
   </sheetData>
+  <printOptions/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>